<commit_message>
add AIFC01-Responsible AI Security
</commit_message>
<xml_diff>
--- a/AIF/AIFC01_Responsible_AI_Security_50.xlsx
+++ b/AIF/AIFC01_Responsible_AI_Security_50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OTHER\AWS\aws-project\AIF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7786B07-82DC-42A6-BC78-DC7BC58D192E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C68691C6-35EA-4A72-AC1F-000977A81465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -208,12 +208,30 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -243,11 +261,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -555,9 +576,14 @@
   <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="95.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="5" width="61.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="0" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="71.85546875" customWidth="1"/>
+    <col min="2" max="2" width="34.5703125" customWidth="1"/>
+    <col min="3" max="3" width="61.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="41.140625" customWidth="1"/>
+    <col min="5" max="5" width="44" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" customWidth="1"/>
+    <col min="7" max="7" width="61.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -590,7 +616,7 @@
       <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C2" t="s">
@@ -602,7 +628,7 @@
       <c r="E2" t="s">
         <v>34</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="4" t="s">
         <v>47</v>
       </c>
       <c r="G2" t="s">
@@ -616,7 +642,7 @@
       <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>29</v>
       </c>
       <c r="C3" t="s">
@@ -628,7 +654,7 @@
       <c r="E3" t="s">
         <v>32</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="4" t="s">
         <v>47</v>
       </c>
       <c r="G3" t="s">
@@ -645,13 +671,13 @@
       <c r="B4" t="s">
         <v>30</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="3" t="s">
         <v>34</v>
       </c>
       <c r="D4" t="s">
         <v>31</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="2" t="s">
         <v>43</v>
       </c>
       <c r="F4" t="s">
@@ -677,10 +703,10 @@
       <c r="D5" t="s">
         <v>32</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="4" t="s">
         <v>49</v>
       </c>
       <c r="G5" t="s">
@@ -697,7 +723,7 @@
       <c r="B6" t="s">
         <v>28</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>33</v>
       </c>
       <c r="D6" t="s">
@@ -706,7 +732,7 @@
       <c r="E6" t="s">
         <v>30</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="4" t="s">
         <v>48</v>
       </c>
       <c r="G6" t="s">
@@ -726,13 +752,13 @@
       <c r="C7" t="s">
         <v>43</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="2" t="s">
         <v>39</v>
       </c>
       <c r="E7" t="s">
         <v>40</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="4" t="s">
         <v>50</v>
       </c>
       <c r="G7" t="s">
@@ -755,10 +781,10 @@
       <c r="D8" t="s">
         <v>33</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="4" t="s">
         <v>49</v>
       </c>
       <c r="G8" t="s">
@@ -781,7 +807,7 @@
       <c r="D9" t="s">
         <v>31</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="3" t="s">
         <v>44</v>
       </c>
       <c r="F9" t="s">
@@ -801,13 +827,13 @@
       <c r="B10" t="s">
         <v>34</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="2" t="s">
         <v>28</v>
       </c>
       <c r="D10" t="s">
         <v>33</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="3" t="s">
         <v>32</v>
       </c>
       <c r="F10" t="s">
@@ -830,10 +856,10 @@
       <c r="C11" t="s">
         <v>43</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="2" t="s">
         <v>37</v>
       </c>
       <c r="F11" t="s">
@@ -859,10 +885,10 @@
       <c r="D12" t="s">
         <v>29</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="4" t="s">
         <v>49</v>
       </c>
       <c r="G12" t="s">
@@ -882,10 +908,10 @@
       <c r="C13" t="s">
         <v>36</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="2" t="s">
         <v>40</v>
       </c>
       <c r="F13" t="s">
@@ -905,13 +931,13 @@
       <c r="B14" t="s">
         <v>30</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="2" t="s">
         <v>38</v>
       </c>
       <c r="D14" t="s">
         <v>36</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="3" t="s">
         <v>40</v>
       </c>
       <c r="F14" t="s">
@@ -937,10 +963,10 @@
       <c r="D15" t="s">
         <v>33</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="4" t="s">
         <v>49</v>
       </c>
       <c r="G15" t="s">
@@ -963,10 +989,10 @@
       <c r="D16" t="s">
         <v>28</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="4" t="s">
         <v>47</v>
       </c>
       <c r="G16" t="s">
@@ -980,10 +1006,10 @@
       <c r="A17" t="s">
         <v>23</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="2" t="s">
         <v>37</v>
       </c>
       <c r="D17" t="s">
@@ -1006,10 +1032,10 @@
       <c r="A18" t="s">
         <v>24</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="3" t="s">
         <v>29</v>
       </c>
       <c r="D18" t="s">
@@ -1032,7 +1058,7 @@
       <c r="A19" t="s">
         <v>25</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="3" t="s">
         <v>37</v>
       </c>
       <c r="C19" t="s">
@@ -1041,7 +1067,7 @@
       <c r="D19" t="s">
         <v>39</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="2" t="s">
         <v>41</v>
       </c>
       <c r="F19" t="s">
@@ -1061,7 +1087,7 @@
       <c r="B20" t="s">
         <v>38</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="2" t="s">
         <v>42</v>
       </c>
       <c r="D20" t="s">
@@ -1070,7 +1096,7 @@
       <c r="E20" t="s">
         <v>34</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="4" t="s">
         <v>48</v>
       </c>
       <c r="G20" t="s">
@@ -1090,13 +1116,13 @@
       <c r="C21" t="s">
         <v>38</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="2" t="s">
         <v>44</v>
       </c>
       <c r="E21" t="s">
         <v>45</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="4" t="s">
         <v>50</v>
       </c>
       <c r="G21" t="s">

</xml_diff>